<commit_message>
feat: support Excel metadata rows
</commit_message>
<xml_diff>
--- a/excel/company-a.xlsx
+++ b/excel/company-a.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fltnn\Documents\Codex\2026-07-04\concur-bot-web-sap-concur-1\outputs\concur-maigo-boshi-bot\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3EDAA67-C079-48B0-B32E-C2AA2B97919C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{733DE5E7-4688-444D-94E1-9376719CBE43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="3" xr2:uid="{249C455E-F0B5-406B-89F2-4DE90A0306D5}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{249C455E-F0B5-406B-89F2-4DE90A0306D5}"/>
   </bookViews>
   <sheets>
     <sheet name="01_基本設定" sheetId="8" r:id="rId1"/>
@@ -526,7 +526,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="90">
   <si>
     <t>company_id</t>
   </si>
@@ -574,9 +574,6 @@
   </si>
   <si>
     <t>海外出張費</t>
-  </si>
-  <si>
-    <t>expense_type_id</t>
   </si>
   <si>
     <t>expense_type_name</t>
@@ -784,11 +781,40 @@
     <t>出張時のみ</t>
   </si>
   <si>
-    <t>company-a</t>
+    <t>タクシー</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>A株式会社</t>
+    <t>normal_expense</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>宿泊費</t>
+    <rPh sb="0" eb="3">
+      <t>シュクハクヒ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>サンプル会社</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>必須</t>
+    <rPh sb="0" eb="2">
+      <t>ヒッス</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>任意</t>
+    <rPh sb="0" eb="2">
+      <t>ニンイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>expense_type_id</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -796,7 +822,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -829,13 +855,37 @@
       <family val="3"/>
       <charset val="128"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="游ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="游ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -852,12 +902,27 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -939,6 +1004,98 @@
         <charset val="128"/>
         <scheme val="minor"/>
       </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -996,44 +1153,22 @@
         <charset val="128"/>
         <scheme val="minor"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1514,8 +1649,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{D84F3076-8FA9-4A7A-B033-E1CE7B7151AB}" name="テーブル68910" displayName="テーブル68910" ref="A1:F4" totalsRowShown="0" headerRowDxfId="8">
-  <autoFilter ref="A1:F4" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{D84F3076-8FA9-4A7A-B033-E1CE7B7151AB}" name="テーブル68910" displayName="テーブル68910" ref="A1:F5" totalsRowShown="0" headerRowDxfId="8">
+  <autoFilter ref="A1:F5" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{A203C0B4-DA8B-47FB-AD93-06B65D3DF83A}" name="申請内容"/>
     <tableColumn id="2" xr3:uid="{0FA34334-E5B3-4C7F-AAB6-BB1D856C1D66}" name="出張に関係"/>
@@ -1524,39 +1659,39 @@
     <tableColumn id="5" xr3:uid="{B2CA613B-7973-4F6B-BAC1-8DDED16AE053}" name="案内メッセージ"/>
     <tableColumn id="6" xr3:uid="{F8B1093F-4243-4E80-817E-DA68810823FE}" name="注意事項"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1C076EDE-3A14-44A0-A174-6B7535F7CD49}" name="テーブル1" displayName="テーブル1" ref="A1:D2" totalsRowShown="0" headerRowDxfId="5">
-  <autoFilter ref="A1:D2" xr:uid="{1C076EDE-3A14-44A0-A174-6B7535F7CD49}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1C076EDE-3A14-44A0-A174-6B7535F7CD49}" name="テーブル1" displayName="テーブル1" ref="A1:D3" totalsRowShown="0" headerRowDxfId="5">
+  <autoFilter ref="A1:D3" xr:uid="{1C076EDE-3A14-44A0-A174-6B7535F7CD49}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{AB2A4918-1B3A-444C-8397-B8D718A1DCC8}" name="company_id"/>
     <tableColumn id="2" xr3:uid="{46034CDA-80A5-45B7-80DC-95A945FB539D}" name="company_name"/>
     <tableColumn id="3" xr3:uid="{CBCAC444-C341-4D24-931B-C49BFFF6A1BC}" name="default_policy_id"/>
     <tableColumn id="4" xr3:uid="{6BE79FE3-AE46-4078-9E1B-5F075FEA78FC}" name="language"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B996CD8C-0A29-479E-8E8E-B660E8186F1E}" name="テーブル2" displayName="テーブル2" ref="A1:D3" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:D3" xr:uid="{B996CD8C-0A29-479E-8E8E-B660E8186F1E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B996CD8C-0A29-479E-8E8E-B660E8186F1E}" name="テーブル2" displayName="テーブル2" ref="A1:D4" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:D4" xr:uid="{B996CD8C-0A29-479E-8E8E-B660E8186F1E}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{08666AA1-F4F1-499A-81C6-0435DF1C9F71}" name="policy_id"/>
     <tableColumn id="2" xr3:uid="{9BF64DC3-D358-4442-B417-F2AB3DDFF344}" name="policy_name"/>
     <tableColumn id="3" xr3:uid="{C7CFA628-8409-4030-8785-50BCC4A6B087}" name="enabled"/>
     <tableColumn id="4" xr3:uid="{1CD91DA0-A2B5-41C3-AD12-B194DB856CD7}" name="display_order"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{39899102-F42A-45C7-B14D-05C2499F2811}" name="テーブル3" displayName="テーブル3" ref="A1:E4" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:E4" xr:uid="{39899102-F42A-45C7-B14D-05C2499F2811}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{39899102-F42A-45C7-B14D-05C2499F2811}" name="テーブル3" displayName="テーブル3" ref="A1:E5" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:E5" xr:uid="{39899102-F42A-45C7-B14D-05C2499F2811}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{DFC75CD8-2F06-42D1-80B3-9FF4CB20C500}" name="expense_type_id"/>
     <tableColumn id="2" xr3:uid="{324312A7-D2F2-4928-A9AB-3A204186A333}" name="policy_id"/>
@@ -1564,7 +1699,7 @@
     <tableColumn id="4" xr3:uid="{3F5DE246-2982-4434-AC60-888A6D609BCF}" name="receipt_required"/>
     <tableColumn id="5" xr3:uid="{C01436A9-DF49-469C-9C12-2B45BE55C107}" name="active"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1923,16 +2058,16 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -1976,41 +2111,41 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>80</v>
-      </c>
       <c r="E1" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
         <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D2" t="s">
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
         <v>12</v>
@@ -2022,12 +2157,12 @@
         <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B4" t="s">
         <v>12</v>
@@ -2039,7 +2174,7 @@
         <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -2061,7 +2196,7 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="17.649999999999999"/>
   <cols>
     <col min="1" max="1" width="10.4375" bestFit="1" customWidth="1"/>
@@ -2072,77 +2207,109 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F2" t="s">
-        <v>62</v>
+    </row>
+    <row r="2" spans="1:6" s="1" customFormat="1">
+      <c r="A2" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="A3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="F3" t="s">
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="4" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D4" t="s">
-        <v>73</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="B5" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="F4" t="s">
-        <v>66</v>
-      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B1048576" xr:uid="{8D3BCA68-F94E-4521-A386-BDAD8C1959B9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B1048576" xr:uid="{8D3BCA68-F94E-4521-A386-BDAD8C1959B9}">
       <formula1>"はい"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2158,7 +2325,7 @@
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="17.649999999999999"/>
   <cols>
     <col min="1" max="1" width="15.6875" bestFit="1" customWidth="1"/>
@@ -2168,37 +2335,57 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C2" t="s">
+    <row r="2" spans="1:4" s="1" customFormat="1">
+      <c r="A2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D3" s="4" t="s">
         <v>7</v>
       </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D1048576" xr:uid="{E079D44C-7AEE-4B39-B574-108FF6C7AE21}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:D1048576" xr:uid="{E079D44C-7AEE-4B39-B574-108FF6C7AE21}">
       <formula1>"ja,en"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2216,7 +2403,7 @@
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="17.649999999999999"/>
   <cols>
     <col min="1" max="1" width="16.6875" bestFit="1" customWidth="1"/>
@@ -2226,51 +2413,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
+    <row r="2" spans="1:4" s="1" customFormat="1">
+      <c r="A2" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D2">
+      <c r="D3" s="4">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
+    <row r="4" spans="1:4">
+      <c r="A4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D3">
+      <c r="D4" s="4">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576" xr:uid="{41D1494D-E6A4-4454-9D06-538895B7543A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C3:C1048576" xr:uid="{41D1494D-E6A4-4454-9D06-538895B7543A}">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2288,7 +2489,7 @@
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="17.649999999999999"/>
   <cols>
     <col min="1" max="1" width="17.0625" customWidth="1"/>
@@ -2299,77 +2500,94 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:5" s="1" customFormat="1">
+      <c r="A2" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
+      <c r="B3" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="D3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E3" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E2" t="s">
+      <c r="B4" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="E4" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D3" t="s">
+      <c r="B5" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" t="s">
-        <v>63</v>
-      </c>
-      <c r="D4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="E5" s="4" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D1048576 E2:E1048576" xr:uid="{E9925988-1936-4F72-BF2A-86C37C8061C2}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:E1048576" xr:uid="{E9925988-1936-4F72-BF2A-86C37C8061C2}">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2398,13 +2616,13 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>60</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>11</v>
@@ -2412,13 +2630,13 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
         <v>26</v>
-      </c>
-      <c r="C2" t="s">
-        <v>27</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -2426,13 +2644,13 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
         <v>28</v>
-      </c>
-      <c r="C3" t="s">
-        <v>29</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -2440,13 +2658,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D4">
         <v>3</v>
@@ -2481,102 +2699,102 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>47</v>
-      </c>
       <c r="D1" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" t="s">
         <v>39</v>
       </c>
-      <c r="C2" t="s">
-        <v>40</v>
-      </c>
       <c r="D2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" t="s">
         <v>48</v>
-      </c>
-      <c r="C5" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" t="s">
         <v>50</v>
-      </c>
-      <c r="C6" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" t="s">
         <v>48</v>
-      </c>
-      <c r="C7" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" t="s">
         <v>50</v>
-      </c>
-      <c r="C8" t="s">
-        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -2611,140 +2829,140 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="F1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" t="s">
         <v>40</v>
       </c>
-      <c r="E2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" t="s">
-        <v>41</v>
-      </c>
       <c r="G2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B4">
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G4" t="s">
         <v>43</v>
-      </c>
-      <c r="G4" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B5">
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F5" t="s">
+        <v>64</v>
+      </c>
+      <c r="G5" t="s">
         <v>65</v>
-      </c>
-      <c r="G5" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B6">
         <v>3</v>
       </c>
       <c r="C6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F6" t="s">
+        <v>64</v>
+      </c>
+      <c r="G6" t="s">
         <v>65</v>
-      </c>
-      <c r="G6" t="s">
-        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: complete local company switching
</commit_message>
<xml_diff>
--- a/excel/company-a.xlsx
+++ b/excel/company-a.xlsx
@@ -2363,11 +2363,15 @@
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>86</v>
+      <c r="A3" t="inlineStr" s="4">
+        <is>
+          <t>company-a</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="4">
+        <is>
+          <t>A株式会社</t>
+        </is>
       </c>
       <c r="C3" s="4" t="s">
         <v>6</v>

</xml_diff>